<commit_message>
disabling ev charging UC
</commit_message>
<xml_diff>
--- a/VerveStacks_ZAF_grids_kan/SuppXLS/Scen_TSParameters_ts_40c.xlsx
+++ b/VerveStacks_ZAF_grids_kan/SuppXLS/Scen_TSParameters_ts_40c.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\VerveStacks_ZAF_grids_kan\SuppXLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B14B859F-1EE3-4A61-B7D1-8158B435115E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61DC470E-0BD0-4409-B99B-E7767BA29962}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28898" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ev_charging_uc" sheetId="6" r:id="rId1"/>
@@ -1550,8 +1550,8 @@
     <row r="19" spans="3:14" ht="14.65" thickTop="1" x14ac:dyDescent="0.45"/>
     <row r="21" spans="3:14" ht="17.649999999999999" thickBot="1" x14ac:dyDescent="0.6">
       <c r="H21" s="3" t="str">
-        <f>IF(H23=H24,"Not Required!","~UC_T: LO")</f>
-        <v>~UC_T: LO</v>
+        <f>IF(H23=H24,"Not Required!","~UC_T: N")</f>
+        <v>~UC_T: N</v>
       </c>
     </row>
     <row r="22" spans="3:14" ht="15" thickTop="1" thickBot="1" x14ac:dyDescent="0.5">

</xml_diff>